<commit_message>
#11 :: Update export behavior, added elevation
</commit_message>
<xml_diff>
--- a/backend/lz_template.xlsx
+++ b/backend/lz_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_dev\avtactools\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3B78B7D-F66D-4E63-870B-3AB0495736A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4893739C-F3C3-401C-8EBD-E5C5EE262F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12500" yWindow="1540" windowWidth="22670" windowHeight="17840" xr2:uid="{BDCCC9EE-A8E6-467E-86F7-FCD898600776}"/>
+    <workbookView xWindow="12310" yWindow="2760" windowWidth="22610" windowHeight="15370" xr2:uid="{BDCCC9EE-A8E6-467E-86F7-FCD898600776}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -138,7 +138,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -206,15 +206,21 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -738,22 +744,6 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -766,20 +756,32 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -809,37 +811,34 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -857,13 +856,22 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1277,408 +1285,408 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="20.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="53" t="s">
+      <c r="B1" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53"/>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="52" t="s">
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="49" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="56" t="s">
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="29"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="27"/>
     </row>
     <row r="3" spans="1:10" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="58" t="s">
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="29"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="27"/>
     </row>
     <row r="4" spans="1:10" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="58" t="s">
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
-      <c r="J4" s="29"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="27"/>
     </row>
     <row r="5" spans="1:10" ht="18.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="59" t="s">
+      <c r="A5" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="58" t="s">
+      <c r="B5" s="56"/>
+      <c r="C5" s="56"/>
+      <c r="D5" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58"/>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="58"/>
-      <c r="J5" s="29"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="55"/>
+      <c r="H5" s="55"/>
+      <c r="I5" s="55"/>
+      <c r="J5" s="27"/>
     </row>
     <row r="6" spans="1:10" ht="26" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="24"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="26"/>
+      <c r="A6" s="22"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="24"/>
     </row>
     <row r="7" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="27"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="29"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="27"/>
     </row>
     <row r="8" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="27"/>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="29"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="27"/>
     </row>
     <row r="9" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="27"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="29"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="27"/>
     </row>
     <row r="10" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="27"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="29"/>
+      <c r="A10" s="25"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="27"/>
     </row>
     <row r="11" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="27"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="29"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="27"/>
     </row>
     <row r="12" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="27"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="28"/>
-      <c r="I12" s="28"/>
-      <c r="J12" s="29"/>
+      <c r="A12" s="25"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
+      <c r="J12" s="27"/>
     </row>
     <row r="13" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="27"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="29"/>
+      <c r="A13" s="25"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="27"/>
     </row>
     <row r="14" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="27"/>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="29"/>
+      <c r="A14" s="25"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="27"/>
     </row>
     <row r="15" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="27"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="29"/>
+      <c r="A15" s="25"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="27"/>
     </row>
     <row r="16" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="27"/>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
-      <c r="I16" s="28"/>
-      <c r="J16" s="29"/>
+      <c r="A16" s="25"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="26"/>
+      <c r="J16" s="27"/>
     </row>
     <row r="17" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="27"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="28"/>
-      <c r="J17" s="29"/>
+      <c r="A17" s="25"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="27"/>
     </row>
     <row r="18" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="27"/>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="28"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="29"/>
+      <c r="A18" s="25"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="27"/>
     </row>
     <row r="19" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="27"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="29"/>
+      <c r="A19" s="25"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
+      <c r="J19" s="27"/>
     </row>
     <row r="20" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="27"/>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="29"/>
+      <c r="A20" s="25"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="27"/>
     </row>
     <row r="21" spans="1:10" ht="26" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="30"/>
-      <c r="B21" s="31"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="31"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="31"/>
-      <c r="G21" s="31"/>
-      <c r="H21" s="31"/>
-      <c r="I21" s="31"/>
-      <c r="J21" s="32"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="30"/>
     </row>
     <row r="22" spans="1:10" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="B22" s="34"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E22" s="35" t="s">
+      <c r="E22" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="F22" s="36"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="37" t="s">
+      <c r="F22" s="34"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="I22" s="34"/>
+      <c r="I22" s="32"/>
       <c r="J22" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="38" t="s">
+      <c r="A23" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="39"/>
-      <c r="C23" s="42" t="s">
+      <c r="B23" s="37"/>
+      <c r="C23" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="D23" s="42" t="s">
+      <c r="D23" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="E23" s="44" t="s">
+      <c r="E23" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="46" t="s">
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I23" s="47"/>
-      <c r="J23" s="3" t="s">
+      <c r="I23" s="44"/>
+      <c r="J23" s="58" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="40"/>
-      <c r="B24" s="41"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="50"/>
-      <c r="E24" s="4" t="s">
+      <c r="A24" s="38"/>
+      <c r="B24" s="39"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="47"/>
+      <c r="E24" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F24" s="51" t="s">
+      <c r="F24" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="G24" s="51"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="48"/>
-      <c r="J24" s="5" t="s">
+      <c r="G24" s="48"/>
+      <c r="H24" s="45"/>
+      <c r="I24" s="45"/>
+      <c r="J24" s="10" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="7" t="s">
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="59"/>
+      <c r="E25" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="F25" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="14"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="49"/>
-      <c r="J25" s="8" t="s">
+      <c r="G25" s="12"/>
+      <c r="H25" s="46"/>
+      <c r="I25" s="46"/>
+      <c r="J25" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
-      <c r="J26" s="20"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="18"/>
     </row>
     <row r="27" spans="1:10" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="21"/>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="23"/>
+      <c r="A27" s="19"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20"/>
+      <c r="I27" s="20"/>
+      <c r="J27" s="21"/>
     </row>
     <row r="28" spans="1:10" ht="18.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="B28" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="9" t="s">
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I28" s="10"/>
-      <c r="J28" s="11" t="s">
+      <c r="I28" s="4"/>
+      <c r="J28" s="5" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>